<commit_message>
Initial ALM AI commit Completed recommendation engine and Gemini integration
</commit_message>
<xml_diff>
--- a/ALM_Data.xlsx
+++ b/ALM_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91870\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21563989-9D6E-40D6-9E87-3273DF84AE4F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC9CCC97-C336-42A2-9C88-8F454AAE2B87}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Asset" sheetId="1" r:id="rId1"/>
@@ -23,23 +23,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t>S.No.</t>
   </si>
@@ -71,7 +60,34 @@
     <t>Liability</t>
   </si>
   <si>
-    <t>KRD Bucket</t>
+    <t>0-6</t>
+  </si>
+  <si>
+    <t>7-10</t>
+  </si>
+  <si>
+    <t>11-18</t>
+  </si>
+  <si>
+    <t>19-26</t>
+  </si>
+  <si>
+    <t>27-32</t>
+  </si>
+  <si>
+    <t>33-40</t>
+  </si>
+  <si>
+    <t>&gt;41</t>
+  </si>
+  <si>
+    <t>Bucket</t>
+  </si>
+  <si>
+    <t>Start Year</t>
+  </si>
+  <si>
+    <t>End Year</t>
   </si>
 </sst>
 </file>
@@ -107,10 +123,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -508,7 +525,7 @@
         <v>50</v>
       </c>
       <c r="C8">
-        <v>200000</v>
+        <v>20000</v>
       </c>
       <c r="D8" s="1">
         <v>0.08</v>
@@ -977,7 +994,7 @@
         <v>5.58</v>
       </c>
       <c r="C2">
-        <v>5.53</v>
+        <v>5.59</v>
       </c>
       <c r="D2">
         <v>5.63</v>
@@ -994,7 +1011,7 @@
         <v>6.11</v>
       </c>
       <c r="C3">
-        <v>6.0100000000000007</v>
+        <v>6.13</v>
       </c>
       <c r="D3">
         <v>6.1800000000000006</v>
@@ -1011,7 +1028,7 @@
         <v>6.3</v>
       </c>
       <c r="C4">
-        <v>6.1499999999999995</v>
+        <v>6.33</v>
       </c>
       <c r="D4">
         <v>6.39</v>
@@ -1028,7 +1045,7 @@
         <v>6.5</v>
       </c>
       <c r="C5">
-        <v>6.3</v>
+        <v>6.54</v>
       </c>
       <c r="D5">
         <v>6.61</v>
@@ -1045,7 +1062,7 @@
         <v>6.58</v>
       </c>
       <c r="C6">
-        <v>6.33</v>
+        <v>6.63</v>
       </c>
       <c r="D6">
         <v>6.71</v>
@@ -1062,7 +1079,7 @@
         <v>6.69</v>
       </c>
       <c r="C7">
-        <v>6.3900000000000006</v>
+        <v>6.75</v>
       </c>
       <c r="D7">
         <v>6.8400000000000007</v>
@@ -1079,7 +1096,7 @@
         <v>6.83</v>
       </c>
       <c r="C8">
-        <v>6.48</v>
+        <v>6.9</v>
       </c>
       <c r="D8">
         <v>7</v>
@@ -1096,7 +1113,7 @@
         <v>6.92</v>
       </c>
       <c r="C9">
-        <v>6.52</v>
+        <v>7</v>
       </c>
       <c r="D9">
         <v>7.11</v>
@@ -1113,7 +1130,7 @@
         <v>6.92</v>
       </c>
       <c r="C10">
-        <v>6.47</v>
+        <v>7.01</v>
       </c>
       <c r="D10">
         <v>7.1150000000000002</v>
@@ -1130,7 +1147,7 @@
         <v>6.93</v>
       </c>
       <c r="C11">
-        <v>6.43</v>
+        <v>7.0299999999999994</v>
       </c>
       <c r="D11">
         <v>7.13</v>
@@ -1147,7 +1164,7 @@
         <v>6.99</v>
       </c>
       <c r="C12">
-        <v>6.5200000000000005</v>
+        <v>7.04</v>
       </c>
       <c r="D12">
         <v>7.1950000000000003</v>
@@ -1164,7 +1181,7 @@
         <v>7.14</v>
       </c>
       <c r="C13">
-        <v>6.6999999999999993</v>
+        <v>7.14</v>
       </c>
       <c r="D13">
         <v>7.35</v>
@@ -1181,7 +1198,7 @@
         <v>7.24</v>
       </c>
       <c r="C14">
-        <v>6.83</v>
+        <v>7.19</v>
       </c>
       <c r="D14">
         <v>7.42</v>
@@ -1198,7 +1215,7 @@
         <v>7.29</v>
       </c>
       <c r="C15">
-        <v>6.91</v>
+        <v>7.19</v>
       </c>
       <c r="D15">
         <v>7.44</v>
@@ -1215,7 +1232,7 @@
         <v>7.38</v>
       </c>
       <c r="C16">
-        <v>7.03</v>
+        <v>7.2299999999999995</v>
       </c>
       <c r="D16">
         <v>7.5</v>
@@ -1232,7 +1249,7 @@
         <v>7.46</v>
       </c>
       <c r="C17">
-        <v>7.1400000000000006</v>
+        <v>7.36</v>
       </c>
       <c r="D17">
         <v>7.55</v>
@@ -1249,7 +1266,7 @@
         <v>7.55</v>
       </c>
       <c r="C18">
-        <v>7.26</v>
+        <v>7.5</v>
       </c>
       <c r="D18">
         <v>7.6099999999999994</v>
@@ -1266,7 +1283,7 @@
         <v>7.63</v>
       </c>
       <c r="C19">
-        <v>7.37</v>
+        <v>7.63</v>
       </c>
       <c r="D19">
         <v>7.66</v>
@@ -1283,7 +1300,7 @@
         <v>7.69</v>
       </c>
       <c r="C20">
-        <v>7.4600000000000009</v>
+        <v>7.74</v>
       </c>
       <c r="D20">
         <v>7.69</v>
@@ -1300,7 +1317,7 @@
         <v>7.74</v>
       </c>
       <c r="C21">
-        <v>7.54</v>
+        <v>7.84</v>
       </c>
       <c r="D21">
         <v>7.71</v>
@@ -1317,7 +1334,7 @@
         <v>7.77</v>
       </c>
       <c r="C22">
-        <v>7.6</v>
+        <v>7.89</v>
       </c>
       <c r="D22">
         <v>8.0250000000000004</v>
@@ -1334,7 +1351,7 @@
         <v>7.78</v>
       </c>
       <c r="C23">
-        <v>7.6400000000000006</v>
+        <v>7.92</v>
       </c>
       <c r="D23">
         <v>8.0050000000000008</v>
@@ -1351,7 +1368,7 @@
         <v>7.78</v>
       </c>
       <c r="C24">
-        <v>7.6700000000000008</v>
+        <v>7.94</v>
       </c>
       <c r="D24">
         <v>7.9750000000000014</v>
@@ -1368,7 +1385,7 @@
         <v>7.77</v>
       </c>
       <c r="C25">
-        <v>7.6899999999999995</v>
+        <v>7.9499999999999993</v>
       </c>
       <c r="D25">
         <v>7.9350000000000005</v>
@@ -1385,7 +1402,7 @@
         <v>7.77</v>
       </c>
       <c r="C26">
-        <v>7.72</v>
+        <v>7.97</v>
       </c>
       <c r="D26">
         <v>7.9050000000000002</v>
@@ -1402,7 +1419,7 @@
         <v>7.77</v>
       </c>
       <c r="C27">
-        <v>7.75</v>
+        <v>7.9899999999999993</v>
       </c>
       <c r="D27">
         <v>7.875</v>
@@ -1419,7 +1436,7 @@
         <v>7.78</v>
       </c>
       <c r="C28">
-        <v>7.79</v>
+        <v>8.02</v>
       </c>
       <c r="D28">
         <v>7.8550000000000013</v>
@@ -1436,7 +1453,7 @@
         <v>7.8</v>
       </c>
       <c r="C29">
-        <v>7.84</v>
+        <v>8.06</v>
       </c>
       <c r="D29">
         <v>7.8450000000000006</v>
@@ -1453,7 +1470,7 @@
         <v>7.84</v>
       </c>
       <c r="C30">
-        <v>7.91</v>
+        <v>8.1199999999999992</v>
       </c>
       <c r="D30">
         <v>7.8550000000000004</v>
@@ -1470,7 +1487,7 @@
         <v>7.88</v>
       </c>
       <c r="C31">
-        <v>7.98</v>
+        <v>8.18</v>
       </c>
       <c r="D31">
         <v>7.8650000000000011</v>
@@ -1487,7 +1504,7 @@
         <v>7.94</v>
       </c>
       <c r="C32">
-        <v>8.07</v>
+        <v>8.26</v>
       </c>
       <c r="D32">
         <v>7.8950000000000014</v>
@@ -1504,7 +1521,7 @@
         <v>8.01</v>
       </c>
       <c r="C33">
-        <v>8.17</v>
+        <v>8.35</v>
       </c>
       <c r="D33">
         <v>7.9350000000000005</v>
@@ -1521,7 +1538,7 @@
         <v>8.08</v>
       </c>
       <c r="C34">
-        <v>8.27</v>
+        <v>8.44</v>
       </c>
       <c r="D34">
         <v>7.955000000000001</v>
@@ -1538,7 +1555,7 @@
         <v>8.14</v>
       </c>
       <c r="C35">
-        <v>8.3600000000000012</v>
+        <v>8.4700000000000006</v>
       </c>
       <c r="D35">
         <v>7.9650000000000016</v>
@@ -1555,7 +1572,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="C36">
-        <v>8.4499999999999993</v>
+        <v>8.5</v>
       </c>
       <c r="D36">
         <v>7.9749999999999996</v>
@@ -1572,7 +1589,7 @@
         <v>8.23</v>
       </c>
       <c r="C37">
-        <v>8.5100000000000016</v>
+        <v>8.5</v>
       </c>
       <c r="D37">
         <v>7.955000000000001</v>
@@ -1589,7 +1606,7 @@
         <v>8.25</v>
       </c>
       <c r="C38">
-        <v>8.56</v>
+        <v>8.49</v>
       </c>
       <c r="D38">
         <v>7.9250000000000007</v>
@@ -1606,7 +1623,7 @@
         <v>8.23</v>
       </c>
       <c r="C39">
-        <v>8.57</v>
+        <v>8.4400000000000013</v>
       </c>
       <c r="D39">
         <v>7.8550000000000013</v>
@@ -1623,7 +1640,7 @@
         <v>8.17</v>
       </c>
       <c r="C40">
-        <v>8.5400000000000009</v>
+        <v>8.35</v>
       </c>
       <c r="D40">
         <v>7.745000000000001</v>
@@ -1640,7 +1657,7 @@
         <v>8.08</v>
       </c>
       <c r="C41">
-        <v>8.48</v>
+        <v>8.23</v>
       </c>
       <c r="D41">
         <v>7.6050000000000013</v>
@@ -1657,7 +1674,7 @@
         <v>8.01</v>
       </c>
       <c r="C42">
-        <v>8.44</v>
+        <v>8.129999999999999</v>
       </c>
       <c r="D42">
         <v>7.5550000000000006</v>
@@ -1674,7 +1691,7 @@
         <v>7.97</v>
       </c>
       <c r="C43">
-        <v>8.43</v>
+        <v>8.06</v>
       </c>
       <c r="D43">
         <v>7.535000000000001</v>
@@ -1691,7 +1708,7 @@
         <v>7.95</v>
       </c>
       <c r="C44">
-        <v>8.4400000000000013</v>
+        <v>8.01</v>
       </c>
       <c r="D44">
         <v>7.535000000000001</v>
@@ -1708,7 +1725,7 @@
         <v>7.97</v>
       </c>
       <c r="C45">
-        <v>8.49</v>
+        <v>8.0499999999999989</v>
       </c>
       <c r="D45">
         <v>7.5750000000000011</v>
@@ -1725,7 +1742,7 @@
         <v>8</v>
       </c>
       <c r="C46">
-        <v>8.5500000000000007</v>
+        <v>8.1</v>
       </c>
       <c r="D46">
         <v>7.6250000000000009</v>
@@ -1742,7 +1759,7 @@
         <v>8.07</v>
       </c>
       <c r="C47">
-        <v>8.65</v>
+        <v>8.19</v>
       </c>
       <c r="D47">
         <v>7.7150000000000016</v>
@@ -1759,7 +1776,7 @@
         <v>8.14</v>
       </c>
       <c r="C48">
-        <v>8.7500000000000018</v>
+        <v>8.2800000000000011</v>
       </c>
       <c r="D48">
         <v>7.8050000000000015</v>
@@ -1776,7 +1793,7 @@
         <v>8.24</v>
       </c>
       <c r="C49">
-        <v>8.8800000000000008</v>
+        <v>8.4</v>
       </c>
       <c r="D49">
         <v>7.9250000000000016</v>
@@ -1793,7 +1810,7 @@
         <v>8.3699999999999992</v>
       </c>
       <c r="C50">
-        <v>9.0399999999999991</v>
+        <v>8.5499999999999989</v>
       </c>
       <c r="D50">
         <v>8.0750000000000011</v>
@@ -1810,7 +1827,7 @@
         <v>8.52</v>
       </c>
       <c r="C51">
-        <v>9.2200000000000006</v>
+        <v>8.7199999999999989</v>
       </c>
       <c r="D51">
         <v>8.245000000000001</v>
@@ -1827,50 +1844,95 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D98185B4-3C18-455A-AB95-6BED797C014E}">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2">
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3">
+        <v>7</v>
+      </c>
+      <c r="C3">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>11</v>
+      </c>
+      <c r="C4">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>19</v>
+      </c>
+      <c r="C5">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6">
+        <v>27</v>
+      </c>
+      <c r="C6">
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7">
+        <v>33</v>
+      </c>
+      <c r="C7">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>99999</v>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8">
+        <v>41</v>
+      </c>
+      <c r="C8">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1880,6 +1942,24 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<Klassify>
+  <SNO>1</SNO>
+  <KDate>2026-07-31 19:16:36</KDate>
+  <Classification>INTERNAL</Classification>
+  <Subclassification/>
+  <HostName>MLI2XQQMZ3</HostName>
+  <Domain_User>MAXLIFE/a.hom6005</Domain_User>
+  <IPAdd>11.114.28.229</IPAdd>
+  <FilePath>https://maxlifeinsurance-my.sharepoint.com/personal/abhishek_14_axismaxlife_com/Documents/Desktop/ALM_Data.xlsx</FilePath>
+  <KID>00FF1C780959639211221962553851</KID>
+  <UniqueName/>
+  <Suggested/>
+  <Justification/>
+  <KlassifyGUID>09de4e4e-a5d1-4fbe-a975-84b94a80b507</KlassifyGUID>
+</Klassify>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <Klassify>
   <SNO>2</SNO>
   <KDate>2026-07-31 23:27:37</KDate>
@@ -1897,32 +1977,14 @@
 </Klassify>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<Klassify>
-  <SNO>1</SNO>
-  <KDate>2026-07-31 19:16:36</KDate>
-  <Classification>INTERNAL</Classification>
-  <Subclassification/>
-  <HostName>MLI2XQQMZ3</HostName>
-  <Domain_User>MAXLIFE/a.hom6005</Domain_User>
-  <IPAdd>11.114.28.229</IPAdd>
-  <FilePath>https://maxlifeinsurance-my.sharepoint.com/personal/abhishek_14_axismaxlife_com/Documents/Desktop/ALM_Data.xlsx</FilePath>
-  <KID>00FF1C780959639211221962553851</KID>
-  <UniqueName/>
-  <Suggested/>
-  <Justification/>
-  <KlassifyGUID>09de4e4e-a5d1-4fbe-a975-84b94a80b507</KlassifyGUID>
-</Klassify>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5CB8BF2-A206-476A-A121-094155B994E7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0AFDBBFE-539E-4748-9FA8-5C4A710D5E38}">
   <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0AFDBBFE-539E-4748-9FA8-5C4A710D5E38}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5CB8BF2-A206-476A-A121-094155B994E7}">
   <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>
</xml_diff>